<commit_message>
Fix bad date entry in phenology Dookie2025
</commit_message>
<xml_diff>
--- a/Tests/Validation/Wheat/UoM_WheatProject/Dookie2025_Observed.xlsx
+++ b/Tests/Validation/Wheat/UoM_WheatProject/Dookie2025_Observed.xlsx
@@ -16631,7 +16631,7 @@
         <v>93</v>
       </c>
       <c r="B548" t="s">
-        <v>94</v>
+        <v>22</v>
       </c>
       <c r="C548"/>
       <c r="D548"/>
@@ -16646,13 +16646,13 @@
       <c r="M548"/>
       <c r="N548"/>
       <c r="O548"/>
-      <c r="P548"/>
+      <c r="P548" t="n">
+        <v>18.5</v>
+      </c>
       <c r="Q548"/>
       <c r="R548"/>
       <c r="S548"/>
-      <c r="T548" t="n">
-        <v>3</v>
-      </c>
+      <c r="T548"/>
       <c r="U548"/>
     </row>
     <row r="549">
@@ -16660,7 +16660,7 @@
         <v>93</v>
       </c>
       <c r="B549" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C549"/>
       <c r="D549"/>
@@ -16675,13 +16675,13 @@
       <c r="M549"/>
       <c r="N549"/>
       <c r="O549"/>
-      <c r="P549" t="n">
-        <v>18.5</v>
-      </c>
+      <c r="P549"/>
       <c r="Q549"/>
       <c r="R549"/>
       <c r="S549"/>
-      <c r="T549"/>
+      <c r="T549" t="n">
+        <v>3</v>
+      </c>
       <c r="U549"/>
     </row>
     <row r="550">
@@ -20488,7 +20488,7 @@
         <v>106</v>
       </c>
       <c r="B681" t="s">
-        <v>94</v>
+        <v>22</v>
       </c>
       <c r="C681"/>
       <c r="D681"/>
@@ -20503,13 +20503,13 @@
       <c r="M681"/>
       <c r="N681"/>
       <c r="O681"/>
-      <c r="P681"/>
+      <c r="P681" t="n">
+        <v>12.25</v>
+      </c>
       <c r="Q681"/>
       <c r="R681"/>
       <c r="S681"/>
-      <c r="T681" t="n">
-        <v>3</v>
-      </c>
+      <c r="T681"/>
       <c r="U681"/>
     </row>
     <row r="682">
@@ -20517,7 +20517,7 @@
         <v>106</v>
       </c>
       <c r="B682" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C682"/>
       <c r="D682"/>
@@ -20532,13 +20532,13 @@
       <c r="M682"/>
       <c r="N682"/>
       <c r="O682"/>
-      <c r="P682" t="n">
-        <v>12.25</v>
-      </c>
+      <c r="P682"/>
       <c r="Q682"/>
       <c r="R682"/>
       <c r="S682"/>
-      <c r="T682"/>
+      <c r="T682" t="n">
+        <v>3</v>
+      </c>
       <c r="U682"/>
     </row>
     <row r="683">
@@ -26346,7 +26346,7 @@
         <v>112</v>
       </c>
       <c r="B883" t="s">
-        <v>94</v>
+        <v>22</v>
       </c>
       <c r="C883"/>
       <c r="D883"/>
@@ -26361,13 +26361,13 @@
       <c r="M883"/>
       <c r="N883"/>
       <c r="O883"/>
-      <c r="P883"/>
+      <c r="P883" t="n">
+        <v>11.5</v>
+      </c>
       <c r="Q883"/>
       <c r="R883"/>
       <c r="S883"/>
-      <c r="T883" t="n">
-        <v>3</v>
-      </c>
+      <c r="T883"/>
       <c r="U883"/>
     </row>
     <row r="884">
@@ -26375,7 +26375,7 @@
         <v>112</v>
       </c>
       <c r="B884" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C884"/>
       <c r="D884"/>
@@ -26390,13 +26390,13 @@
       <c r="M884"/>
       <c r="N884"/>
       <c r="O884"/>
-      <c r="P884" t="n">
-        <v>11.5</v>
-      </c>
+      <c r="P884"/>
       <c r="Q884"/>
       <c r="R884"/>
       <c r="S884"/>
-      <c r="T884"/>
+      <c r="T884" t="n">
+        <v>3</v>
+      </c>
       <c r="U884"/>
     </row>
     <row r="885">
@@ -28405,7 +28405,7 @@
         <v>115</v>
       </c>
       <c r="B954" t="s">
-        <v>94</v>
+        <v>22</v>
       </c>
       <c r="C954"/>
       <c r="D954"/>
@@ -28420,13 +28420,13 @@
       <c r="M954"/>
       <c r="N954"/>
       <c r="O954"/>
-      <c r="P954"/>
+      <c r="P954" t="n">
+        <v>17.75</v>
+      </c>
       <c r="Q954"/>
       <c r="R954"/>
       <c r="S954"/>
-      <c r="T954" t="n">
-        <v>3</v>
-      </c>
+      <c r="T954"/>
       <c r="U954"/>
     </row>
     <row r="955">
@@ -28449,13 +28449,13 @@
       <c r="M955"/>
       <c r="N955"/>
       <c r="O955"/>
-      <c r="P955" t="n">
-        <v>17.75</v>
-      </c>
+      <c r="P955"/>
       <c r="Q955"/>
       <c r="R955"/>
       <c r="S955"/>
-      <c r="T955"/>
+      <c r="T955" t="n">
+        <v>3</v>
+      </c>
       <c r="U955"/>
     </row>
     <row r="956">
@@ -30406,7 +30406,7 @@
         <v>116</v>
       </c>
       <c r="B1023" t="s">
-        <v>94</v>
+        <v>22</v>
       </c>
       <c r="C1023"/>
       <c r="D1023"/>
@@ -30421,13 +30421,13 @@
       <c r="M1023"/>
       <c r="N1023"/>
       <c r="O1023"/>
-      <c r="P1023"/>
+      <c r="P1023" t="n">
+        <v>13</v>
+      </c>
       <c r="Q1023"/>
       <c r="R1023"/>
       <c r="S1023"/>
-      <c r="T1023" t="n">
-        <v>3</v>
-      </c>
+      <c r="T1023"/>
       <c r="U1023"/>
     </row>
     <row r="1024">
@@ -30435,7 +30435,7 @@
         <v>116</v>
       </c>
       <c r="B1024" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C1024"/>
       <c r="D1024"/>
@@ -30450,13 +30450,13 @@
       <c r="M1024"/>
       <c r="N1024"/>
       <c r="O1024"/>
-      <c r="P1024" t="n">
-        <v>13</v>
-      </c>
+      <c r="P1024"/>
       <c r="Q1024"/>
       <c r="R1024"/>
       <c r="S1024"/>
-      <c r="T1024"/>
+      <c r="T1024" t="n">
+        <v>3</v>
+      </c>
       <c r="U1024"/>
     </row>
     <row r="1025">
@@ -36409,7 +36409,7 @@
         <v>123</v>
       </c>
       <c r="B1230" t="s">
-        <v>94</v>
+        <v>22</v>
       </c>
       <c r="C1230"/>
       <c r="D1230"/>
@@ -36424,13 +36424,13 @@
       <c r="M1230"/>
       <c r="N1230"/>
       <c r="O1230"/>
-      <c r="P1230"/>
+      <c r="P1230" t="n">
+        <v>14.25</v>
+      </c>
       <c r="Q1230"/>
       <c r="R1230"/>
       <c r="S1230"/>
-      <c r="T1230" t="n">
-        <v>3</v>
-      </c>
+      <c r="T1230"/>
       <c r="U1230"/>
     </row>
     <row r="1231">
@@ -36438,7 +36438,7 @@
         <v>123</v>
       </c>
       <c r="B1231" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C1231"/>
       <c r="D1231"/>
@@ -36453,13 +36453,13 @@
       <c r="M1231"/>
       <c r="N1231"/>
       <c r="O1231"/>
-      <c r="P1231" t="n">
-        <v>14.25</v>
-      </c>
+      <c r="P1231"/>
       <c r="Q1231"/>
       <c r="R1231"/>
       <c r="S1231"/>
-      <c r="T1231"/>
+      <c r="T1231" t="n">
+        <v>3</v>
+      </c>
       <c r="U1231"/>
     </row>
     <row r="1232">
@@ -38352,7 +38352,7 @@
         <v>125</v>
       </c>
       <c r="B1297" t="s">
-        <v>94</v>
+        <v>22</v>
       </c>
       <c r="C1297"/>
       <c r="D1297"/>
@@ -38367,13 +38367,13 @@
       <c r="M1297"/>
       <c r="N1297"/>
       <c r="O1297"/>
-      <c r="P1297"/>
+      <c r="P1297" t="n">
+        <v>16.25</v>
+      </c>
       <c r="Q1297"/>
       <c r="R1297"/>
       <c r="S1297"/>
-      <c r="T1297" t="n">
-        <v>3</v>
-      </c>
+      <c r="T1297"/>
       <c r="U1297"/>
     </row>
     <row r="1298">
@@ -38381,7 +38381,7 @@
         <v>125</v>
       </c>
       <c r="B1298" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C1298"/>
       <c r="D1298"/>
@@ -38396,13 +38396,13 @@
       <c r="M1298"/>
       <c r="N1298"/>
       <c r="O1298"/>
-      <c r="P1298" t="n">
-        <v>16.25</v>
-      </c>
+      <c r="P1298"/>
       <c r="Q1298"/>
       <c r="R1298"/>
       <c r="S1298"/>
-      <c r="T1298"/>
+      <c r="T1298" t="n">
+        <v>3</v>
+      </c>
       <c r="U1298"/>
     </row>
     <row r="1299">
@@ -42325,7 +42325,7 @@
         <v>127</v>
       </c>
       <c r="B1434" t="s">
-        <v>94</v>
+        <v>22</v>
       </c>
       <c r="C1434"/>
       <c r="D1434"/>
@@ -42340,13 +42340,13 @@
       <c r="M1434"/>
       <c r="N1434"/>
       <c r="O1434"/>
-      <c r="P1434"/>
+      <c r="P1434" t="n">
+        <v>12.5</v>
+      </c>
       <c r="Q1434"/>
       <c r="R1434"/>
       <c r="S1434"/>
-      <c r="T1434" t="n">
-        <v>3</v>
-      </c>
+      <c r="T1434"/>
       <c r="U1434"/>
     </row>
     <row r="1435">
@@ -42354,7 +42354,7 @@
         <v>127</v>
       </c>
       <c r="B1435" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C1435"/>
       <c r="D1435"/>
@@ -42369,13 +42369,13 @@
       <c r="M1435"/>
       <c r="N1435"/>
       <c r="O1435"/>
-      <c r="P1435" t="n">
-        <v>12.5</v>
-      </c>
+      <c r="P1435"/>
       <c r="Q1435"/>
       <c r="R1435"/>
       <c r="S1435"/>
-      <c r="T1435"/>
+      <c r="T1435" t="n">
+        <v>3</v>
+      </c>
       <c r="U1435"/>
     </row>
     <row r="1436">

</xml_diff>

<commit_message>
Fix Diikie 2025 unit of grain size
</commit_message>
<xml_diff>
--- a/Tests/Validation/Wheat/UoM_WheatProject/Dookie2025_Observed.xlsx
+++ b/Tests/Validation/Wheat/UoM_WheatProject/Dookie2025_Observed.xlsx
@@ -2276,7 +2276,7 @@
       <c r="D53"/>
       <c r="E53"/>
       <c r="F53" t="n">
-        <v>34.8375</v>
+        <v>0.0348375</v>
       </c>
       <c r="G53"/>
       <c r="H53"/>
@@ -4016,7 +4016,7 @@
       <c r="D113"/>
       <c r="E113"/>
       <c r="F113" t="n">
-        <v>28.6</v>
+        <v>0.0286</v>
       </c>
       <c r="G113"/>
       <c r="H113"/>
@@ -5756,7 +5756,7 @@
       <c r="D173"/>
       <c r="E173"/>
       <c r="F173" t="n">
-        <v>30.6</v>
+        <v>0.0306</v>
       </c>
       <c r="G173"/>
       <c r="H173"/>
@@ -7496,7 +7496,7 @@
       <c r="D233"/>
       <c r="E233"/>
       <c r="F233" t="n">
-        <v>29.3375</v>
+        <v>0.0293375</v>
       </c>
       <c r="G233"/>
       <c r="H233"/>
@@ -9178,7 +9178,7 @@
       <c r="D291"/>
       <c r="E291"/>
       <c r="F291" t="n">
-        <v>30.2</v>
+        <v>0.0302</v>
       </c>
       <c r="G291"/>
       <c r="H291"/>
@@ -10860,7 +10860,7 @@
       <c r="D349"/>
       <c r="E349"/>
       <c r="F349" t="n">
-        <v>32.0375</v>
+        <v>0.0320375</v>
       </c>
       <c r="G349"/>
       <c r="H349"/>
@@ -12542,7 +12542,7 @@
       <c r="D407"/>
       <c r="E407"/>
       <c r="F407" t="n">
-        <v>32.3375</v>
+        <v>0.0323375</v>
       </c>
       <c r="G407"/>
       <c r="H407"/>
@@ -14224,7 +14224,7 @@
       <c r="D465"/>
       <c r="E465"/>
       <c r="F465" t="n">
-        <v>34.2875</v>
+        <v>0.0342875</v>
       </c>
       <c r="G465"/>
       <c r="H465"/>
@@ -16109,7 +16109,7 @@
       <c r="D530"/>
       <c r="E530"/>
       <c r="F530" t="n">
-        <v>33.4625</v>
+        <v>0.0334625</v>
       </c>
       <c r="G530"/>
       <c r="H530"/>
@@ -18052,7 +18052,7 @@
       <c r="D597"/>
       <c r="E597"/>
       <c r="F597" t="n">
-        <v>34.6875</v>
+        <v>0.0346875</v>
       </c>
       <c r="G597"/>
       <c r="H597"/>
@@ -19966,7 +19966,7 @@
       <c r="D663"/>
       <c r="E663"/>
       <c r="F663" t="n">
-        <v>31.875</v>
+        <v>0.031875</v>
       </c>
       <c r="G663"/>
       <c r="H663"/>
@@ -21909,7 +21909,7 @@
       <c r="D730"/>
       <c r="E730"/>
       <c r="F730" t="n">
-        <v>34.0875</v>
+        <v>0.0340875</v>
       </c>
       <c r="G730"/>
       <c r="H730"/>
@@ -23910,7 +23910,7 @@
       <c r="D799"/>
       <c r="E799"/>
       <c r="F799" t="n">
-        <v>32.2375</v>
+        <v>0.0322375</v>
       </c>
       <c r="G799"/>
       <c r="H799"/>
@@ -25824,7 +25824,7 @@
       <c r="D865"/>
       <c r="E865"/>
       <c r="F865" t="n">
-        <v>28.7875</v>
+        <v>0.0287875</v>
       </c>
       <c r="G865"/>
       <c r="H865"/>
@@ -27883,7 +27883,7 @@
       <c r="D936"/>
       <c r="E936"/>
       <c r="F936" t="n">
-        <v>30.0875</v>
+        <v>0.0300875</v>
       </c>
       <c r="G936"/>
       <c r="H936"/>
@@ -29884,7 +29884,7 @@
       <c r="D1005"/>
       <c r="E1005"/>
       <c r="F1005" t="n">
-        <v>28.3</v>
+        <v>0.0283</v>
       </c>
       <c r="G1005"/>
       <c r="H1005"/>
@@ -31885,7 +31885,7 @@
       <c r="D1074"/>
       <c r="E1074"/>
       <c r="F1074" t="n">
-        <v>27.375</v>
+        <v>0.027375</v>
       </c>
       <c r="G1074"/>
       <c r="H1074"/>
@@ -33915,7 +33915,7 @@
       <c r="D1144"/>
       <c r="E1144"/>
       <c r="F1144" t="n">
-        <v>38.825</v>
+        <v>0.038825</v>
       </c>
       <c r="G1144"/>
       <c r="H1144"/>
@@ -35887,7 +35887,7 @@
       <c r="D1212"/>
       <c r="E1212"/>
       <c r="F1212" t="n">
-        <v>35.025</v>
+        <v>0.035025</v>
       </c>
       <c r="G1212"/>
       <c r="H1212"/>
@@ -37830,7 +37830,7 @@
       <c r="D1279"/>
       <c r="E1279"/>
       <c r="F1279" t="n">
-        <v>28.0375</v>
+        <v>0.0280375</v>
       </c>
       <c r="G1279"/>
       <c r="H1279"/>
@@ -39918,7 +39918,7 @@
       <c r="D1351"/>
       <c r="E1351"/>
       <c r="F1351" t="n">
-        <v>28.15</v>
+        <v>0.02815</v>
       </c>
       <c r="G1351"/>
       <c r="H1351"/>
@@ -41803,7 +41803,7 @@
       <c r="D1416"/>
       <c r="E1416"/>
       <c r="F1416" t="n">
-        <v>34.0875</v>
+        <v>0.0340875</v>
       </c>
       <c r="G1416"/>
       <c r="H1416"/>
@@ -43688,7 +43688,7 @@
       <c r="D1481"/>
       <c r="E1481"/>
       <c r="F1481" t="n">
-        <v>29.6625</v>
+        <v>0.0296625</v>
       </c>
       <c r="G1481"/>
       <c r="H1481"/>
@@ -45573,7 +45573,7 @@
       <c r="D1546"/>
       <c r="E1546"/>
       <c r="F1546" t="n">
-        <v>33.875</v>
+        <v>0.033875</v>
       </c>
       <c r="G1546"/>
       <c r="H1546"/>

</xml_diff>